<commit_message>
fix sliders to use actual input data
Signed-off-by: ChinmayeRaju <chinmayeraju2510@gmail.com>
</commit_message>
<xml_diff>
--- a/questionnaire_data/truth_or_thought_research_data.xlsx
+++ b/questionnaire_data/truth_or_thought_research_data.xlsx
@@ -920,7 +920,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:H4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1040,6 +1040,34 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>exit_1756136902439_y582cefg</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>2025-08-25T15:48:22.439Z</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>exit</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="n">
+        <v>5</v>
+      </c>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1051,7 +1079,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H10"/>
+  <dimension ref="A1:H14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="33" customWidth="1" min="1" max="1"/>
@@ -1271,6 +1299,74 @@
       <c r="H10" t="inlineStr">
         <is>
           <t>dasda</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>session_1756135869711_br0xt3v1l</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>2025-08-25T15:31:09.711Z</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>session</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>session_1756136083415_55ikx6xrr</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>2025-08-25T15:34:43.415Z</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>session</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>session_1756136313290_pypu2set1</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>2025-08-25T15:38:33.290Z</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>session</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>session_1756136428583_r12618prk</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>2025-08-25T15:40:28.583Z</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>session</t>
         </is>
       </c>
     </row>
@@ -1356,11 +1452,6 @@
           <t>b46f74a4-ef8d-4af2-b870-ae4ee56feebe</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
fix post pre questionnaires
Signed-off-by: ChinmayeRaju <chinmayeraju2510@gmail.com>
</commit_message>
<xml_diff>
--- a/questionnaire_data/truth_or_thought_research_data.xlsx
+++ b/questionnaire_data/truth_or_thought_research_data.xlsx
@@ -1056,12 +1056,9 @@
           <t>exit</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr"/>
-      <c r="E4" t="inlineStr"/>
       <c r="F4" t="n">
         <v>5</v>
       </c>
-      <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr">
         <is>
           <t>no</t>
@@ -1079,7 +1076,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H14"/>
+  <dimension ref="A1:H15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="33" customWidth="1" min="1" max="1"/>
@@ -1367,6 +1364,32 @@
       <c r="C14" t="inlineStr">
         <is>
           <t>session</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>session_1756149833206_q23asgx6z</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>2025-08-25T19:23:53.206Z</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>session</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr"/>
+      <c r="E15" t="inlineStr"/>
+      <c r="F15" t="inlineStr"/>
+      <c r="G15" t="inlineStr"/>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
     </row>

</xml_diff>